<commit_message>
Standardize radio model to 8T8R across all models and set author to OLIVER TUNGOL in all Excel properties
</commit_message>
<xml_diff>
--- a/2026-09-25_Revised_Models/FWA_Metric_to_Source_Mapping_2024.xlsx
+++ b/2026-09-25_Revised_Models/FWA_Metric_to_Source_Mapping_2024.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metric to Source Mapping (2024)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Datasets (2024)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Metric to Source Mapping (2024)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Source Datasets (2024)" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1271,6 +1271,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>

</xml_diff>